<commit_message>
fix: agrega columna client_code a la carga masiva de comprobantes
Actualiza la plantilla descargable (xlsx) y el texto de ayuda para
incluir client_code, requerido en clientes holding para desambiguar
la empresa correcta (ver PRD_fix_disambiguacion_comprobantes_holding.md).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/invoice_attachments_template.xlsx
+++ b/public/templates/invoice_attachments_template.xlsx
@@ -1,73 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet sheetId="1" name="comprobantes" state="visible" r:id="rId4"/>
+    <sheet name="comprobantes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>number</t>
-  </si>
-  <si>
-    <t>nombre_archivo</t>
-  </si>
-  <si>
-    <t>codigo_deudor</t>
-  </si>
-  <si>
-    <t>tipo_documento</t>
-  </si>
-  <si>
-    <t>12345</t>
-  </si>
-  <si>
-    <t>comprobante_transferencia_12345.pdf</t>
-  </si>
-  <si>
-    <t>D-001</t>
-  </si>
-  <si>
-    <t>INVOICE</t>
-  </si>
-  <si>
-    <t>12346</t>
-  </si>
-  <si>
-    <t>comprobante_transferencia_12346.pdf</t>
-  </si>
-  <si>
-    <t>D-002</t>
-  </si>
-  <si>
-    <t>CREDIT_NOTE</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <family val="2"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -86,24 +46,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -428,60 +447,104 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="1" width="15" style="1" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col width="15" customWidth="1" style="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
+    <row r="1" customFormat="1" s="2">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>nombre_archivo</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>codigo_deudor</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>tipo_documento</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>client_code</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>comprobante_transferencia_12345.pdf</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>D-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>INVOICE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>EMP-001</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>12346</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>comprobante_transferencia_12346.pdf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>D-002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CREDIT_NOTE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EMP-002</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>